<commit_message>
Distinguish Midcheck, quiz lessons, semester Credit and year-end Exam
</commit_message>
<xml_diff>
--- a/frontend/templates/grammar-semester-topics.xlsx
+++ b/frontend/templates/grammar-semester-topics.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lesson topics" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson topics" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lesson topics'!$A$1:$E$19</definedName>
@@ -560,7 +560,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Consolidation Test</t>
+          <t>Midcheck</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -606,12 +606,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>IMT-1 Quiz and revision</t>
+          <t>IMT-1 Quiz presentations</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>imt</t>
+          <t>lesson</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -619,7 +619,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>IMT-1 quiz; follow-up exercises before Assessment Test 1.</t>
+          <t>Students present their own quizzes; follow-up exercises before Assessment Test 1.</t>
         </is>
       </c>
     </row>
@@ -859,12 +859,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Final credit</t>
+          <t>Credit</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>credit</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -880,7 +880,7 @@
   <autoFilter ref="A1:E19"/>
   <dataValidations count="1">
     <dataValidation sqref="C2:C121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"lesson,test,imt,extra"</formula1>
+      <formula1>"lesson,test,credit,exam,imt,extra"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>